<commit_message>
Editorial layout rework, impact scenarios, Public Sans
</commit_message>
<xml_diff>
--- a/AI model energy calculator.xlsx
+++ b/AI model energy calculator.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Assumptions" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Calculator" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Scenarios" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Impact" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" name="GridList" vbProcedure="false">Assumptions!$A$5:$A$10</definedName>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="203">
   <si>
     <t xml:space="preserve">AI model energy calculator: MVP, task-first</t>
   </si>
@@ -568,13 +569,85 @@
   </si>
   <si>
     <t xml:space="preserve">Carbon multiple, India vs Norway</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Donor impact scenarios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What a $1M eco-labeling project could plausibly influence. Impact scales with the share of global inference traffic that routing integrations, procurement standards, and disclosure pressure reach.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parameters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global AI inference electricity, 2026 (GWh)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IEA: AI data centers ~155 TWh in 2025, +30%/yr, ~60% inference share. Confidence C.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wholesale electricity price ($/MWh)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicative global blend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grid carbon intensity (kgCO2e/kWh)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ember world average</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project cost ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First-year grant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scenario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Influenced share of inference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energy saved on influenced slice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GWh saved per year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$M saved per year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ktCO2e avoided per year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$ per tCO2e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annual leverage (savings / cost)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conservative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Central</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ambitious</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reading the table: the Central case assumes integrations and standards reach 0.5% of global inference traffic and cut its energy in half, consistent with the per-task savings this workbook demonstrates. Even the Conservative case returns roughly 3x the grant annually; the abatement cost compares favorably with typical climate philanthropy at $10-100 per tCO2e.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Why platform-layer leverage is plausible: OpenRouter routes 20T+ tokens weekly and its mix already shifted heavily toward cheap models on price alone; Google processed 3.2 quadrillion tokens in May 2026; ~97% of Anthropic API usage is automation-dominant. One routing integration moves more traffic than any number of individual user choices.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
     <numFmt numFmtId="166" formatCode="#,##0"/>
@@ -585,6 +658,7 @@
     <numFmt numFmtId="171" formatCode="0%"/>
     <numFmt numFmtId="172" formatCode="0.0%"/>
     <numFmt numFmtId="173" formatCode="0.0"/>
+    <numFmt numFmtId="174" formatCode="0.0\x"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -730,8 +804,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -751,19 +829,19 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -771,19 +849,99 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -791,31 +949,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -823,7 +961,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -831,19 +969,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1102,94 +1232,94 @@
   <dimension ref="A1:A20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="110"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="3" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="3" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1212,505 +1342,505 @@
   <dimension ref="A1:P12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="11" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="11" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+    <row r="1" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="P1" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="D2" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="I2" s="5" t="n">
+      <c r="I2" s="6" t="n">
         <v>33</v>
       </c>
-      <c r="J2" s="5" t="n">
+      <c r="J2" s="6" t="n">
         <v>85</v>
       </c>
-      <c r="K2" s="6" t="n">
+      <c r="K2" s="7" t="n">
         <v>12.345</v>
       </c>
-      <c r="L2" s="6" t="n">
+      <c r="L2" s="7" t="n">
         <v>21.311</v>
       </c>
-      <c r="M2" s="6" t="n">
+      <c r="M2" s="7" t="n">
         <v>30.278</v>
       </c>
-      <c r="N2" s="6" t="n">
+      <c r="N2" s="7" t="n">
         <f aca="false">L2/1.5</f>
         <v>14.2073333333333</v>
       </c>
-      <c r="O2" s="5" t="n">
+      <c r="O2" s="6" t="n">
         <v>0.34</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="P2" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="D3" s="7" t="n">
+      <c r="D3" s="8" t="n">
         <v>39</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="I3" s="7" t="n">
+      <c r="I3" s="8" t="n">
         <v>29</v>
       </c>
-      <c r="J3" s="7" t="n">
+      <c r="J3" s="8" t="n">
         <v>71</v>
       </c>
-      <c r="K3" s="8" t="n">
+      <c r="K3" s="9" t="n">
         <v>2.339</v>
       </c>
-      <c r="L3" s="8" t="n">
+      <c r="L3" s="9" t="n">
         <v>3.65</v>
       </c>
-      <c r="M3" s="8" t="n">
+      <c r="M3" s="9" t="n">
         <v>4.961</v>
       </c>
-      <c r="N3" s="8" t="n">
+      <c r="N3" s="9" t="n">
         <f aca="false">L3/1.5</f>
         <v>2.43333333333333</v>
       </c>
-      <c r="O3" s="7" t="n">
+      <c r="O3" s="8" t="n">
         <v>0.34</v>
       </c>
-      <c r="P3" s="7" t="s">
+      <c r="P3" s="8" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="I4" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="J4" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="K4" s="6" t="n">
+      <c r="K4" s="7" t="n">
         <v>0.537</v>
       </c>
-      <c r="L4" s="6" t="n">
+      <c r="L4" s="7" t="n">
         <v>0.634</v>
       </c>
-      <c r="M4" s="6" t="n">
+      <c r="M4" s="7" t="n">
         <v>0.732</v>
       </c>
-      <c r="N4" s="6" t="n">
+      <c r="N4" s="7" t="n">
         <f aca="false">L4/1.5</f>
         <v>0.422666666666667</v>
       </c>
-      <c r="O4" s="5" t="n">
+      <c r="O4" s="6" t="n">
         <v>0.34</v>
       </c>
-      <c r="P4" s="5" t="s">
+      <c r="P4" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="8" t="n">
         <v>61</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="8" t="n">
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="9" t="n">
         <v>10.9</v>
       </c>
-      <c r="L5" s="8" t="n">
+      <c r="L5" s="9" t="n">
         <v>14.46</v>
       </c>
-      <c r="M5" s="8" t="n">
+      <c r="M5" s="9" t="n">
         <v>18.1</v>
       </c>
-      <c r="N5" s="8" t="n">
+      <c r="N5" s="9" t="n">
         <f aca="false">L5/1.5</f>
         <v>9.64</v>
       </c>
-      <c r="O5" s="7" t="n">
+      <c r="O5" s="8" t="n">
         <v>0.3</v>
       </c>
-      <c r="P5" s="7" t="s">
+      <c r="P5" s="8" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="6" t="n">
         <v>43</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="I6" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="J6" s="5" t="n">
+      <c r="J6" s="6" t="n">
         <v>78</v>
       </c>
-      <c r="K6" s="6" t="n">
+      <c r="K6" s="7" t="n">
         <v>7.633</v>
       </c>
-      <c r="L6" s="6" t="n">
+      <c r="L6" s="7" t="n">
         <v>9.79</v>
       </c>
-      <c r="M6" s="6" t="n">
+      <c r="M6" s="7" t="n">
         <v>11.947</v>
       </c>
-      <c r="N6" s="6" t="n">
+      <c r="N6" s="7" t="n">
         <f aca="false">L6/1.5</f>
         <v>6.52666666666667</v>
       </c>
-      <c r="O6" s="5" t="n">
+      <c r="O6" s="6" t="n">
         <v>0.3</v>
       </c>
-      <c r="P6" s="5" t="s">
+      <c r="P6" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="8" t="n">
         <v>37</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="I7" s="7" t="n">
+      <c r="I7" s="8" t="n">
         <v>27</v>
       </c>
-      <c r="J7" s="7" t="n">
+      <c r="J7" s="8" t="n">
         <v>55</v>
       </c>
-      <c r="K7" s="8" t="n">
+      <c r="K7" s="9" t="n">
         <v>2.099</v>
       </c>
-      <c r="L7" s="8" t="n">
+      <c r="L7" s="9" t="n">
         <v>11.199</v>
       </c>
-      <c r="M7" s="8" t="n">
+      <c r="M7" s="9" t="n">
         <v>20.3</v>
       </c>
-      <c r="N7" s="8" t="n">
+      <c r="N7" s="9" t="n">
         <f aca="false">L7/1.5</f>
         <v>7.466</v>
       </c>
-      <c r="O7" s="7" t="n">
+      <c r="O7" s="8" t="n">
         <v>0.3</v>
       </c>
-      <c r="P7" s="7" t="s">
+      <c r="P7" s="8" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="6" t="n">
         <v>35</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="I8" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="J8" s="5" t="n">
+      <c r="J8" s="6" t="n">
         <v>54</v>
       </c>
-      <c r="K8" s="6" t="n">
+      <c r="K8" s="7" t="n">
         <v>2.25</v>
       </c>
-      <c r="L8" s="6" t="n">
+      <c r="L8" s="7" t="n">
         <v>3.155</v>
       </c>
-      <c r="M8" s="6" t="n">
+      <c r="M8" s="7" t="n">
         <v>4.06</v>
       </c>
-      <c r="N8" s="6" t="n">
+      <c r="N8" s="7" t="n">
         <f aca="false">L8/1.5</f>
         <v>2.10333333333333</v>
       </c>
-      <c r="O8" s="5" t="n">
+      <c r="O8" s="6" t="n">
         <v>0.231</v>
       </c>
-      <c r="P8" s="5" t="s">
+      <c r="P8" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="8" t="n">
         <v>27</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="I9" s="7" t="n">
+      <c r="I9" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="J9" s="7" t="n">
+      <c r="J9" s="8" t="n">
         <v>32</v>
       </c>
-      <c r="K9" s="8" t="n">
+      <c r="K9" s="9" t="n">
         <v>1.135</v>
       </c>
-      <c r="L9" s="8" t="n">
+      <c r="L9" s="9" t="n">
         <v>2.314</v>
       </c>
-      <c r="M9" s="8" t="n">
+      <c r="M9" s="9" t="n">
         <v>3.494</v>
       </c>
-      <c r="N9" s="8" t="n">
+      <c r="N9" s="9" t="n">
         <f aca="false">L9/1.5</f>
         <v>1.54266666666667</v>
       </c>
-      <c r="O9" s="7" t="n">
+      <c r="O9" s="8" t="n">
         <v>0.231</v>
       </c>
-      <c r="P9" s="7" t="s">
+      <c r="P9" s="8" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="9"/>
-    </row>
-    <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="s">
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+    </row>
+    <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1735,184 +1865,184 @@
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="4" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="4" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="72"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+    <row r="1" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="10" t="n">
+      <c r="B2" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="10" t="n">
+      <c r="E2" s="11" t="n">
         <v>150</v>
       </c>
-      <c r="F2" s="10" t="n">
+      <c r="F2" s="11" t="n">
         <v>700</v>
       </c>
-      <c r="G2" s="10" t="n">
+      <c r="G2" s="11" t="n">
         <v>1500</v>
       </c>
-      <c r="H2" s="10" t="n">
+      <c r="H2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="I2" s="8" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="B3" s="10" t="n">
+      <c r="B3" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="10" t="n">
+      <c r="E3" s="11" t="n">
         <v>800</v>
       </c>
-      <c r="F3" s="10" t="n">
+      <c r="F3" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="G3" s="10" t="n">
+      <c r="G3" s="11" t="n">
         <v>4000</v>
       </c>
-      <c r="H3" s="10" t="n">
+      <c r="H3" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="8" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="B4" s="10" t="n">
+      <c r="B4" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="E4" s="10" t="n">
+      <c r="E4" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="F4" s="10" t="n">
+      <c r="F4" s="11" t="n">
         <v>4500</v>
       </c>
-      <c r="G4" s="10" t="n">
+      <c r="G4" s="11" t="n">
         <v>8000</v>
       </c>
-      <c r="H4" s="10" t="n">
+      <c r="H4" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="I4" s="8" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="11" t="n">
         <v>33</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="E5" s="11" t="n">
         <v>1000</v>
       </c>
-      <c r="F5" s="10" t="n">
+      <c r="F5" s="11" t="n">
         <v>1500</v>
       </c>
-      <c r="G5" s="10" t="n">
+      <c r="G5" s="11" t="n">
         <v>2500</v>
       </c>
-      <c r="H5" s="10" t="n">
+      <c r="H5" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1937,206 +2067,206 @@
   <dimension ref="A1:D23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="52"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="11" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="12" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="13" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="14" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="15" t="s">
+      <c r="B5" s="15"/>
+      <c r="C5" s="16" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B6" s="14" t="n">
+      <c r="B6" s="15" t="n">
         <v>0.369</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="16" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="B7" s="14" t="n">
+      <c r="B7" s="15" t="n">
         <v>0.213</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="16" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B8" s="15" t="n">
         <v>0.028</v>
       </c>
-      <c r="C8" s="15" t="s">
+      <c r="C8" s="16" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="15" t="n">
         <v>0.713</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="16" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="B10" s="14" t="n">
+      <c r="B10" s="15" t="n">
         <v>0.481</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="16" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="D13" s="14" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="B14" s="16" t="n">
+      <c r="B14" s="17" t="n">
         <v>29.6</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="D14" s="15" t="s">
+      <c r="D14" s="16" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="B15" s="17" t="n">
+      <c r="B15" s="18" t="n">
         <v>0.17</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="16" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="18" t="n">
         <v>0.012</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="D16" s="15" t="s">
+      <c r="D16" s="16" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="B17" s="16" t="n">
+      <c r="B17" s="17" t="n">
         <v>10791</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D17" s="16" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="12" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="B20" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="C20" s="13" t="s">
+      <c r="C20" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="D20" s="13" t="s">
+      <c r="D20" s="14" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="B21" s="10" t="n">
+      <c r="B21" s="11" t="n">
         <v>2500000000</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="D21" s="15" t="s">
+      <c r="D21" s="16" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="18" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="19" t="s">
         <v>111</v>
       </c>
     </row>
@@ -2159,360 +2289,360 @@
   <dimension ref="A1:E42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="5" min="5" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="5" min="5" style="1" width="13"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="11" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="12" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="19" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="13" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="21" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="20" t="s">
+      <c r="E6" s="21" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="20" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="11" t="n">
         <v>1000</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="20" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="20" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13"/>
-      <c r="B12" s="13" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="14"/>
+      <c r="B12" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="14" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="B13" s="21" t="n">
+      <c r="B13" s="22" t="n">
         <f aca="false">INDEX(Models!$D$2:$D$9,MATCH($B$6,Models!$B$2:$B$9,0))</f>
         <v>45</v>
       </c>
-      <c r="C13" s="21" t="n">
+      <c r="C13" s="22" t="n">
         <f aca="false">INDEX(Models!$D$2:$D$9,MATCH($B$7,Models!$B$2:$B$9,0))</f>
         <v>27</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="7" t="str">
+      <c r="B14" s="8" t="str">
         <f aca="false">INDEX(Models!$F$2:$F$9,MATCH($B$6,Models!$B$2:$B$9,0))</f>
         <v>high</v>
       </c>
-      <c r="C14" s="7" t="str">
+      <c r="C14" s="8" t="str">
         <f aca="false">INDEX(Models!$F$2:$F$9,MATCH($B$7,Models!$B$2:$B$9,0))</f>
         <v>none</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="B15" s="22" t="n">
+      <c r="B15" s="23" t="n">
         <f aca="false">IF(B14="none",INDEX(Tasks!$E$2:$E$5,MATCH($B$5,Tasks!$A$2:$A$5,0)),IF(B14="medium",INDEX(Tasks!$F$2:$F$5,MATCH($B$5,Tasks!$A$2:$A$5,0)),INDEX(Tasks!$G$2:$G$5,MATCH($B$5,Tasks!$A$2:$A$5,0))))</f>
         <v>4000</v>
       </c>
-      <c r="C15" s="22" t="n">
+      <c r="C15" s="23" t="n">
         <f aca="false">IF(C14="none",INDEX(Tasks!$E$2:$E$5,MATCH($B$5,Tasks!$A$2:$A$5,0)),IF(C14="medium",INDEX(Tasks!$F$2:$F$5,MATCH($B$5,Tasks!$A$2:$A$5,0)),INDEX(Tasks!$G$2:$G$5,MATCH($B$5,Tasks!$A$2:$A$5,0))))</f>
         <v>800</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="B16" s="21" t="n">
+      <c r="B16" s="22" t="n">
         <f aca="false">INDEX(Tasks!$H$2:$H$5,MATCH($B$5,Tasks!$A$2:$A$5,0))</f>
         <v>1</v>
       </c>
-      <c r="C16" s="21" t="n">
+      <c r="C16" s="22" t="n">
         <f aca="false">INDEX(Tasks!$H$2:$H$5,MATCH($B$5,Tasks!$A$2:$A$5,0))</f>
         <v>1</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="B17" s="22" t="n">
+      <c r="B17" s="23" t="n">
         <f aca="false">B15*B16</f>
         <v>4000</v>
       </c>
-      <c r="C17" s="22" t="n">
+      <c r="C17" s="23" t="n">
         <f aca="false">C15*C16</f>
         <v>800</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="B18" s="8" t="n">
+      <c r="B18" s="9" t="n">
         <f aca="false">INDEX(Models!$L$2:$L$9,MATCH($B$6,Models!$B$2:$B$9,0))/1500*B17</f>
         <v>56.8293333333333</v>
       </c>
-      <c r="C18" s="8" t="n">
+      <c r="C18" s="9" t="n">
         <f aca="false">INDEX(Models!$L$2:$L$9,MATCH($B$7,Models!$B$2:$B$9,0))/1500*C17</f>
         <v>1.23413333333333</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="B19" s="8" t="n">
+      <c r="B19" s="9" t="n">
         <f aca="false">INDEX(Models!$K$2:$K$9,MATCH($B$6,Models!$B$2:$B$9,0))/1500*B17</f>
         <v>32.92</v>
       </c>
-      <c r="C19" s="8" t="n">
+      <c r="C19" s="9" t="n">
         <f aca="false">INDEX(Models!$K$2:$K$9,MATCH($B$7,Models!$B$2:$B$9,0))/1500*C17</f>
         <v>0.605333333333333</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="B20" s="8" t="n">
+      <c r="B20" s="9" t="n">
         <f aca="false">INDEX(Models!$M$2:$M$9,MATCH($B$6,Models!$B$2:$B$9,0))/1500*B17</f>
         <v>80.7413333333333</v>
       </c>
-      <c r="C20" s="8" t="n">
+      <c r="C20" s="9" t="n">
         <f aca="false">INDEX(Models!$M$2:$M$9,MATCH($B$7,Models!$B$2:$B$9,0))/1500*C17</f>
         <v>1.86346666666667</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B21" s="7" t="str">
+      <c r="B21" s="8" t="str">
         <f aca="false">IF(OR(B13&lt;INDEX(Tasks!$B$2:$B$5,MATCH($B$5,Tasks!$A$2:$A$5,0)),AND(INDEX(Tasks!$C$2:$C$5,MATCH($B$5,Tasks!$A$2:$A$5,0))="yes",INDEX(Models!$G$2:$G$9,MATCH($B$6,Models!$B$2:$B$9,0))="no"),AND(INDEX(Tasks!$D$2:$D$5,MATCH($B$5,Tasks!$A$2:$A$5,0))="yes",INDEX(Models!$H$2:$H$9,MATCH($B$6,Models!$B$2:$B$9,0))="no")),"Warning: likely not capable of this task","OK")</f>
         <v>OK</v>
       </c>
-      <c r="C21" s="7" t="str">
+      <c r="C21" s="8" t="str">
         <f aca="false">IF(OR(C13&lt;INDEX(Tasks!$B$2:$B$5,MATCH($B$5,Tasks!$A$2:$A$5,0)),AND(INDEX(Tasks!$C$2:$C$5,MATCH($B$5,Tasks!$A$2:$A$5,0))="yes",INDEX(Models!$G$2:$G$9,MATCH($B$7,Models!$B$2:$B$9,0))="no"),AND(INDEX(Tasks!$D$2:$D$5,MATCH($B$5,Tasks!$A$2:$A$5,0))="yes",INDEX(Models!$H$2:$H$9,MATCH($B$7,Models!$B$2:$B$9,0))="no")),"Warning: likely not capable of this task","OK")</f>
         <v>OK</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="B22" s="23" t="n">
+      <c r="B22" s="24" t="n">
         <f aca="false">MAX(0.35,MIN(0.97,0.6+0.02*(B13-INDEX(Tasks!$B$2:$B$5,MATCH($B$5,Tasks!$A$2:$A$5,0)))))</f>
         <v>0.97</v>
       </c>
-      <c r="C22" s="23" t="n">
+      <c r="C22" s="24" t="n">
         <f aca="false">MAX(0.35,MIN(0.97,0.6+0.02*(C13-INDEX(Tasks!$B$2:$B$5,MATCH($B$5,Tasks!$A$2:$A$5,0)))))</f>
         <v>0.78</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="B23" s="8" t="n">
+      <c r="B23" s="9" t="n">
         <f aca="false">IF($B$10="Yes",B18/B22,B18)</f>
         <v>56.8293333333333</v>
       </c>
-      <c r="C23" s="8" t="n">
+      <c r="C23" s="9" t="n">
         <f aca="false">IF($B$10="Yes",C18/C22,C18)</f>
         <v>1.23413333333333</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="B24" s="24" t="n">
+      <c r="B24" s="25" t="n">
         <f aca="false">B23*$B$8/1000</f>
         <v>56.8293333333333</v>
       </c>
-      <c r="C24" s="24" t="n">
+      <c r="C24" s="25" t="n">
         <f aca="false">C23*$B$8/1000</f>
         <v>1.23413333333333</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="B25" s="22" t="n">
+      <c r="B25" s="23" t="n">
         <f aca="false">B24*12</f>
         <v>681.952</v>
       </c>
-      <c r="C25" s="22" t="n">
+      <c r="C25" s="23" t="n">
         <f aca="false">C24*12</f>
         <v>14.8096</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="12" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="13" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="B28" s="8" t="n">
+      <c r="B28" s="9" t="n">
         <f aca="false">B23-C23</f>
         <v>55.5952</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="B29" s="25" t="n">
+      <c r="B29" s="26" t="n">
         <f aca="false">IF(B23=0,"",(B23-C23)/B23)</f>
         <v>0.978283515555347</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="B30" s="22" t="n">
+      <c r="B30" s="23" t="n">
         <f aca="false">B25-C25</f>
         <v>667.1424</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="B31" s="22" t="n">
+      <c r="B31" s="23" t="n">
         <f aca="false">(B19-C20)*$B$8*12/1000</f>
         <v>372.6784</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="B32" s="22" t="n">
+      <c r="B32" s="23" t="n">
         <f aca="false">(B20-C19)*$B$8*12/1000</f>
         <v>961.632</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="12" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="13" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B35" s="24" t="n">
+      <c r="B35" s="25" t="n">
         <f aca="false">ABS(B30)/Assumptions!$B$14</f>
         <v>22.5385945945946</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="7" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="B36" s="22" t="n">
+      <c r="B36" s="23" t="n">
         <f aca="false">ABS(B30)/Assumptions!$B$15</f>
         <v>3924.36705882353</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="7" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="B37" s="22" t="n">
+      <c r="B37" s="23" t="n">
         <f aca="false">ABS(B30)/Assumptions!$B$16</f>
         <v>55595.2</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="12" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="13" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="7" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="B40" s="22" t="n">
+      <c r="B40" s="23" t="n">
         <f aca="false">IF($B$9="Host default",B25*INDEX(Models!$O$2:$O$9,MATCH($B$6,Models!$B$2:$B$9,0))-C25*INDEX(Models!$O$2:$O$9,MATCH($B$7,Models!$B$2:$B$9,0)),B30*INDEX(Assumptions!$B$5:$B$10,MATCH($B$9,Assumptions!$A$5:$A$10,0)))</f>
         <v>228.4426624</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="9" t="s">
+      <c r="A42" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="B42" s="9"/>
-      <c r="C42" s="9"/>
+      <c r="B42" s="10"/>
+      <c r="C42" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2558,327 +2688,327 @@
   <dimension ref="A1:E42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="11" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="12" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="13" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="19" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="20" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="14" t="s">
         <v>151</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="14" t="s">
         <v>152</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="14" t="s">
         <v>153</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="14" t="s">
         <v>154</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="14" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="str">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="str">
         <f aca="false">Tasks!$A$2</f>
         <v>Classify or extract</v>
       </c>
-      <c r="B8" s="26" t="n">
+      <c r="B8" s="27" t="n">
         <v>0.55</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="9" t="n">
         <f aca="false">INDEX(Models!$L$2:$L$9,MATCH($B$5,Models!$B$2:$B$9,0))/1500*IF(INDEX(Models!$F$2:$F$9,MATCH($B$5,Models!$B$2:$B$9,0))="none",Tasks!$E$2,IF(INDEX(Models!$F$2:$F$9,MATCH($B$5,Models!$B$2:$B$9,0))="medium",Tasks!$F$2,Tasks!$G$2))*Tasks!$H$2</f>
         <v>21.311</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="9" t="n">
         <f aca="false">INDEX(Models!$L$2:$L$9,MATCH($C8,Models!$B$2:$B$9,0))/1500*IF(INDEX(Models!$F$2:$F$9,MATCH($C8,Models!$B$2:$B$9,0))="none",Tasks!$E$2,IF(INDEX(Models!$F$2:$F$9,MATCH($C8,Models!$B$2:$B$9,0))="medium",Tasks!$F$2,Tasks!$G$2))*Tasks!$H$2</f>
         <v>0.0634</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="str">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="str">
         <f aca="false">Tasks!$A$3</f>
         <v>Draft an email or summary</v>
       </c>
-      <c r="B9" s="26" t="n">
+      <c r="B9" s="27" t="n">
         <v>0.3</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="9" t="n">
         <f aca="false">INDEX(Models!$L$2:$L$9,MATCH($B$5,Models!$B$2:$B$9,0))/1500*IF(INDEX(Models!$F$2:$F$9,MATCH($B$5,Models!$B$2:$B$9,0))="none",Tasks!$E$3,IF(INDEX(Models!$F$2:$F$9,MATCH($B$5,Models!$B$2:$B$9,0))="medium",Tasks!$F$3,Tasks!$G$3))*Tasks!$H$3</f>
         <v>56.8293333333333</v>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="9" t="n">
         <f aca="false">INDEX(Models!$L$2:$L$9,MATCH($C9,Models!$B$2:$B$9,0))/1500*IF(INDEX(Models!$F$2:$F$9,MATCH($C9,Models!$B$2:$B$9,0))="none",Tasks!$E$3,IF(INDEX(Models!$F$2:$F$9,MATCH($C9,Models!$B$2:$B$9,0))="medium",Tasks!$F$3,Tasks!$G$3))*Tasks!$H$3</f>
         <v>1.23413333333333</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="str">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="str">
         <f aca="false">Tasks!$A$4</f>
         <v>Complex analysis</v>
       </c>
-      <c r="B10" s="26" t="n">
+      <c r="B10" s="27" t="n">
         <v>0.12</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="9" t="n">
         <f aca="false">INDEX(Models!$L$2:$L$9,MATCH($B$5,Models!$B$2:$B$9,0))/1500*IF(INDEX(Models!$F$2:$F$9,MATCH($B$5,Models!$B$2:$B$9,0))="none",Tasks!$E$4,IF(INDEX(Models!$F$2:$F$9,MATCH($B$5,Models!$B$2:$B$9,0))="medium",Tasks!$F$4,Tasks!$G$4))*Tasks!$H$4</f>
         <v>113.658666666667</v>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="9" t="n">
         <f aca="false">INDEX(Models!$L$2:$L$9,MATCH($C10,Models!$B$2:$B$9,0))/1500*IF(INDEX(Models!$F$2:$F$9,MATCH($C10,Models!$B$2:$B$9,0))="none",Tasks!$E$4,IF(INDEX(Models!$F$2:$F$9,MATCH($C10,Models!$B$2:$B$9,0))="medium",Tasks!$F$4,Tasks!$G$4))*Tasks!$H$4</f>
         <v>9.465</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="str">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="str">
         <f aca="false">Tasks!$A$5</f>
         <v>Agentic multi-step job</v>
       </c>
-      <c r="B11" s="26" t="n">
+      <c r="B11" s="27" t="n">
         <v>0.03</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="9" t="n">
         <f aca="false">INDEX(Models!$L$2:$L$9,MATCH($B$5,Models!$B$2:$B$9,0))/1500*IF(INDEX(Models!$F$2:$F$9,MATCH($B$5,Models!$B$2:$B$9,0))="none",Tasks!$E$5,IF(INDEX(Models!$F$2:$F$9,MATCH($B$5,Models!$B$2:$B$9,0))="medium",Tasks!$F$5,Tasks!$G$5))*Tasks!$H$5</f>
         <v>461.738333333333</v>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="9" t="n">
         <f aca="false">INDEX(Models!$L$2:$L$9,MATCH($C11,Models!$B$2:$B$9,0))/1500*IF(INDEX(Models!$F$2:$F$9,MATCH($C11,Models!$B$2:$B$9,0))="none",Tasks!$E$5,IF(INDEX(Models!$F$2:$F$9,MATCH($C11,Models!$B$2:$B$9,0))="medium",Tasks!$F$5,Tasks!$G$5))*Tasks!$H$5</f>
         <v>41.015</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="B13" s="23" t="n">
+      <c r="B13" s="24" t="n">
         <f aca="false">SUM(B8:B11)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="9" t="n">
         <f aca="false">SUMPRODUCT($B$8:$B$11,D8:D11)</f>
         <v>56.26104</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="B15" s="8" t="n">
+      <c r="B15" s="9" t="n">
         <f aca="false">SUMPRODUCT($B$8:$B$11,E8:E11)</f>
         <v>2.77136</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="B16" s="25" t="n">
+      <c r="B16" s="26" t="n">
         <f aca="false">IF(B14=0,"",1-B15/B14)</f>
         <v>0.950741045668548</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="B18" s="26" t="n">
+      <c r="B18" s="27" t="n">
         <v>0.5</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="B19" s="22" t="n">
+      <c r="B19" s="23" t="n">
         <f aca="false">(B14-B15)*B18*Assumptions!$B$21*365/1000000000</f>
         <v>24404.6665</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="s">
         <v>162</v>
       </c>
-      <c r="B20" s="22" t="n">
+      <c r="B20" s="23" t="n">
         <f aca="false">B19*1000000/Assumptions!$B$17</f>
         <v>2261575.9892503</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="B21" s="22" t="n">
+      <c r="B21" s="23" t="n">
         <f aca="false">B19*1000000*Assumptions!$B$10/1000</f>
         <v>11738644.5865</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="12" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="18" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="19" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="B26" s="22" t="n">
+      <c r="B26" s="23" t="n">
         <f aca="false">Assumptions!$B$21</f>
         <v>2500000000</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="B27" s="27" t="n">
+      <c r="B27" s="28" t="n">
         <v>0.01</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="B28" s="19" t="s">
+      <c r="B28" s="20" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="B29" s="19" t="s">
+      <c r="B29" s="20" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="B31" s="7" t="str">
+      <c r="B31" s="8" t="str">
         <f aca="false">TEXT(INDEX(Models!$L$2:$L$9,MATCH($B$28,Models!$B$2:$B$9,0)),"0.00")&amp;" / "&amp;TEXT(INDEX(Models!$L$2:$L$9,MATCH($B$29,Models!$B$2:$B$9,0)),"0.00")</f>
         <v>21.31 / 3.65</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="B32" s="24" t="n">
+      <c r="B32" s="25" t="n">
         <f aca="false">(INDEX(Models!$L$2:$L$9,MATCH($B$28,Models!$B$2:$B$9,0))-INDEX(Models!$L$2:$L$9,MATCH($B$29,Models!$B$2:$B$9,0)))*B26*B27*365/1000000000</f>
         <v>161.156625</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="B33" s="22" t="n">
+      <c r="B33" s="23" t="n">
         <f aca="false">ABS(B32)*1000000/Assumptions!$B$17</f>
         <v>14934.3550180706</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="B34" s="22" t="n">
+      <c r="B34" s="23" t="n">
         <f aca="false">B32*1000000*Assumptions!$B$10/1000</f>
         <v>77516.336625</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="12" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="13" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="7" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B38" s="19" t="s">
+      <c r="B38" s="20" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="7" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="B39" s="22" t="n">
+      <c r="B39" s="23" t="n">
         <f aca="false">INDEX(Models!$L$2:$L$9,MATCH($B$38,Models!$B$2:$B$9,0))*1000000/1000</f>
         <v>9790</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="7" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="B40" s="8" t="n">
+      <c r="B40" s="9" t="n">
         <f aca="false">B39*Assumptions!$B$8/1000</f>
         <v>0.27412</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="7" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="B41" s="8" t="n">
+      <c r="B41" s="9" t="n">
         <f aca="false">B39*Assumptions!$B$9/1000</f>
         <v>6.98027</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="7" t="s">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="8" t="s">
         <v>178</v>
       </c>
-      <c r="B42" s="28" t="n">
+      <c r="B42" s="29" t="n">
         <f aca="false">IF(B40=0,"",B41/B40)</f>
         <v>25.4642857142857</v>
       </c>
@@ -2926,4 +3056,250 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H19"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="30" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="31" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="32" t="s">
+        <v>182</v>
+      </c>
+      <c r="B5" s="33" t="n">
+        <v>120000</v>
+      </c>
+      <c r="C5" s="34" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="32" t="s">
+        <v>184</v>
+      </c>
+      <c r="B6" s="33" t="n">
+        <v>80</v>
+      </c>
+      <c r="C6" s="34" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="32" t="s">
+        <v>186</v>
+      </c>
+      <c r="B7" s="35" t="n">
+        <v>0.481</v>
+      </c>
+      <c r="C7" s="34" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="32" t="s">
+        <v>188</v>
+      </c>
+      <c r="B8" s="33" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="C8" s="34" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="31" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="32" t="s">
+        <v>198</v>
+      </c>
+      <c r="B13" s="36" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="C13" s="37" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D13" s="38" t="n">
+        <f aca="false">$B$5*B13*C13</f>
+        <v>36</v>
+      </c>
+      <c r="E13" s="39" t="n">
+        <f aca="false">D13*$B$6/1000</f>
+        <v>2.88</v>
+      </c>
+      <c r="F13" s="40" t="n">
+        <f aca="false">D13*$B$7</f>
+        <v>17.316</v>
+      </c>
+      <c r="G13" s="41" t="n">
+        <f aca="false">IF(F13=0,"",$B$8/(F13*1000))</f>
+        <v>57.7500577500578</v>
+      </c>
+      <c r="H13" s="42" t="n">
+        <f aca="false">E13*1000000/$B$8</f>
+        <v>2.88</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="32" t="s">
+        <v>199</v>
+      </c>
+      <c r="B14" s="36" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="C14" s="37" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D14" s="38" t="n">
+        <f aca="false">$B$5*B14*C14</f>
+        <v>300</v>
+      </c>
+      <c r="E14" s="39" t="n">
+        <f aca="false">D14*$B$6/1000</f>
+        <v>24</v>
+      </c>
+      <c r="F14" s="40" t="n">
+        <f aca="false">D14*$B$7</f>
+        <v>144.3</v>
+      </c>
+      <c r="G14" s="41" t="n">
+        <f aca="false">IF(F14=0,"",$B$8/(F14*1000))</f>
+        <v>6.93000693000693</v>
+      </c>
+      <c r="H14" s="42" t="n">
+        <f aca="false">E14*1000000/$B$8</f>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="32" t="s">
+        <v>200</v>
+      </c>
+      <c r="B15" s="36" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C15" s="37" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D15" s="38" t="n">
+        <f aca="false">$B$5*B15*C15</f>
+        <v>1680</v>
+      </c>
+      <c r="E15" s="39" t="n">
+        <f aca="false">D15*$B$6/1000</f>
+        <v>134.4</v>
+      </c>
+      <c r="F15" s="40" t="n">
+        <f aca="false">D15*$B$7</f>
+        <v>808.08</v>
+      </c>
+      <c r="G15" s="41" t="n">
+        <f aca="false">IF(F15=0,"",$B$8/(F15*1000))</f>
+        <v>1.23750123750124</v>
+      </c>
+      <c r="H15" s="42" t="n">
+        <f aca="false">E15*1000000/$B$8</f>
+        <v>134.4</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
+    </row>
+    <row r="19" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A19:H19"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>